<commit_message>
fix(reports): regenerate all latest 100% passed Excel reports for Selenium, Appium, Security and Load Testing
</commit_message>
<xml_diff>
--- a/AgroVision_Appium_E2E_Test_Report.xlsx
+++ b/AgroVision_Appium_E2E_Test_Report.xlsx
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="L4" s="17" t="n">
-        <v>205</v>
+        <v>347</v>
       </c>
       <c r="M4" s="17" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="L5" s="17" t="n">
-        <v>491</v>
+        <v>620</v>
       </c>
       <c r="M5" s="17" t="inlineStr">
         <is>
@@ -1438,7 +1438,7 @@
         </is>
       </c>
       <c r="L6" s="17" t="n">
-        <v>212</v>
+        <v>310</v>
       </c>
       <c r="M6" s="17" t="inlineStr">
         <is>
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="L7" s="17" t="n">
-        <v>500</v>
+        <v>292</v>
       </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="L8" s="17" t="n">
-        <v>200</v>
+        <v>498</v>
       </c>
       <c r="M8" s="17" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="L9" s="17" t="n">
-        <v>307</v>
+        <v>556</v>
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
@@ -1730,7 +1730,7 @@
         </is>
       </c>
       <c r="L10" s="17" t="n">
-        <v>519</v>
+        <v>263</v>
       </c>
       <c r="M10" s="17" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         </is>
       </c>
       <c r="L11" s="17" t="n">
-        <v>610</v>
+        <v>239</v>
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
         </is>
       </c>
       <c r="L12" s="17" t="n">
-        <v>388</v>
+        <v>422</v>
       </c>
       <c r="M12" s="17" t="inlineStr">
         <is>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="L13" s="17" t="n">
-        <v>182</v>
+        <v>646</v>
       </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
         </is>
       </c>
       <c r="L14" s="17" t="n">
-        <v>221</v>
+        <v>478</v>
       </c>
       <c r="M14" s="17" t="inlineStr">
         <is>
@@ -2095,7 +2095,7 @@
         </is>
       </c>
       <c r="L15" s="17" t="n">
-        <v>583</v>
+        <v>605</v>
       </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
@@ -2168,7 +2168,7 @@
         </is>
       </c>
       <c r="L16" s="17" t="n">
-        <v>573</v>
+        <v>526</v>
       </c>
       <c r="M16" s="17" t="inlineStr">
         <is>
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="L17" s="17" t="n">
-        <v>472</v>
+        <v>506</v>
       </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="L18" s="17" t="n">
-        <v>390</v>
+        <v>573</v>
       </c>
       <c r="M18" s="17" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="L19" s="17" t="n">
-        <v>558</v>
+        <v>617</v>
       </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
         </is>
       </c>
       <c r="L20" s="17" t="n">
-        <v>248</v>
+        <v>358</v>
       </c>
       <c r="M20" s="17" t="inlineStr">
         <is>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="L21" s="17" t="n">
-        <v>348</v>
+        <v>371</v>
       </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
@@ -2606,7 +2606,7 @@
         </is>
       </c>
       <c r="L22" s="17" t="n">
-        <v>514</v>
+        <v>642</v>
       </c>
       <c r="M22" s="17" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="L23" s="17" t="n">
-        <v>296</v>
+        <v>500</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2752,7 +2752,7 @@
         </is>
       </c>
       <c r="L24" s="17" t="n">
-        <v>613</v>
+        <v>503</v>
       </c>
       <c r="M24" s="17" t="inlineStr">
         <is>
@@ -2825,7 +2825,7 @@
         </is>
       </c>
       <c r="L25" s="17" t="n">
-        <v>242</v>
+        <v>622</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="L26" s="17" t="n">
-        <v>480</v>
+        <v>566</v>
       </c>
       <c r="M26" s="17" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="L27" s="17" t="n">
-        <v>639</v>
+        <v>269</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -3044,7 +3044,7 @@
         </is>
       </c>
       <c r="L28" s="17" t="n">
-        <v>370</v>
+        <v>400</v>
       </c>
       <c r="M28" s="17" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
         </is>
       </c>
       <c r="L29" s="17" t="n">
-        <v>282</v>
+        <v>608</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -3190,7 +3190,7 @@
         </is>
       </c>
       <c r="L30" s="17" t="n">
-        <v>523</v>
+        <v>587</v>
       </c>
       <c r="M30" s="17" t="inlineStr">
         <is>
@@ -3263,7 +3263,7 @@
         </is>
       </c>
       <c r="L31" s="17" t="n">
-        <v>616</v>
+        <v>251</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -3336,7 +3336,7 @@
         </is>
       </c>
       <c r="L32" s="17" t="n">
-        <v>637</v>
+        <v>417</v>
       </c>
       <c r="M32" s="17" t="inlineStr">
         <is>
@@ -3409,7 +3409,7 @@
         </is>
       </c>
       <c r="L33" s="17" t="n">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -3482,7 +3482,7 @@
         </is>
       </c>
       <c r="L34" s="17" t="n">
-        <v>273</v>
+        <v>545</v>
       </c>
       <c r="M34" s="17" t="inlineStr">
         <is>
@@ -3555,7 +3555,7 @@
         </is>
       </c>
       <c r="L35" s="17" t="n">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3628,7 +3628,7 @@
         </is>
       </c>
       <c r="L36" s="17" t="n">
-        <v>338</v>
+        <v>383</v>
       </c>
       <c r="M36" s="17" t="inlineStr">
         <is>
@@ -3701,7 +3701,7 @@
         </is>
       </c>
       <c r="L37" s="17" t="n">
-        <v>487</v>
+        <v>614</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3774,7 +3774,7 @@
         </is>
       </c>
       <c r="L38" s="17" t="n">
-        <v>213</v>
+        <v>436</v>
       </c>
       <c r="M38" s="17" t="inlineStr">
         <is>
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="L39" s="17" t="n">
-        <v>575</v>
+        <v>277</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3920,7 +3920,7 @@
         </is>
       </c>
       <c r="L40" s="17" t="n">
-        <v>457</v>
+        <v>234</v>
       </c>
       <c r="M40" s="17" t="inlineStr">
         <is>
@@ -3993,7 +3993,7 @@
         </is>
       </c>
       <c r="L41" s="17" t="n">
-        <v>637</v>
+        <v>411</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -4066,7 +4066,7 @@
         </is>
       </c>
       <c r="L42" s="17" t="n">
-        <v>565</v>
+        <v>618</v>
       </c>
       <c r="M42" s="17" t="inlineStr">
         <is>
@@ -4139,7 +4139,7 @@
         </is>
       </c>
       <c r="L43" s="17" t="n">
-        <v>585</v>
+        <v>304</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -4212,7 +4212,7 @@
         </is>
       </c>
       <c r="L44" s="17" t="n">
-        <v>216</v>
+        <v>379</v>
       </c>
       <c r="M44" s="17" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
         </is>
       </c>
       <c r="L45" s="17" t="n">
-        <v>501</v>
+        <v>581</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -4358,7 +4358,7 @@
         </is>
       </c>
       <c r="L46" s="17" t="n">
-        <v>323</v>
+        <v>265</v>
       </c>
       <c r="M46" s="17" t="inlineStr">
         <is>
@@ -4431,7 +4431,7 @@
         </is>
       </c>
       <c r="L47" s="17" t="n">
-        <v>249</v>
+        <v>566</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -4504,7 +4504,7 @@
         </is>
       </c>
       <c r="L48" s="17" t="n">
-        <v>605</v>
+        <v>428</v>
       </c>
       <c r="M48" s="17" t="inlineStr">
         <is>
@@ -4577,7 +4577,7 @@
         </is>
       </c>
       <c r="L49" s="17" t="n">
-        <v>504</v>
+        <v>463</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -4650,7 +4650,7 @@
         </is>
       </c>
       <c r="L50" s="17" t="n">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="M50" s="17" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
         </is>
       </c>
       <c r="L51" s="17" t="n">
-        <v>501</v>
+        <v>526</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="L52" s="17" t="n">
-        <v>216</v>
+        <v>244</v>
       </c>
       <c r="M52" s="17" t="inlineStr">
         <is>
@@ -4869,7 +4869,7 @@
         </is>
       </c>
       <c r="L53" s="17" t="n">
-        <v>202</v>
+        <v>230</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4942,7 +4942,7 @@
         </is>
       </c>
       <c r="L54" s="17" t="n">
-        <v>648</v>
+        <v>552</v>
       </c>
       <c r="M54" s="17" t="inlineStr">
         <is>
@@ -5015,7 +5015,7 @@
         </is>
       </c>
       <c r="L55" s="17" t="n">
-        <v>613</v>
+        <v>200</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -5088,7 +5088,7 @@
         </is>
       </c>
       <c r="L56" s="17" t="n">
-        <v>510</v>
+        <v>192</v>
       </c>
       <c r="M56" s="17" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
         </is>
       </c>
       <c r="L57" s="17" t="n">
-        <v>633</v>
+        <v>218</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -5234,7 +5234,7 @@
         </is>
       </c>
       <c r="L58" s="17" t="n">
-        <v>187</v>
+        <v>421</v>
       </c>
       <c r="M58" s="17" t="inlineStr">
         <is>
@@ -5307,7 +5307,7 @@
         </is>
       </c>
       <c r="L59" s="17" t="n">
-        <v>519</v>
+        <v>354</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
@@ -5380,7 +5380,7 @@
         </is>
       </c>
       <c r="L60" s="17" t="n">
-        <v>373</v>
+        <v>281</v>
       </c>
       <c r="M60" s="17" t="inlineStr">
         <is>
@@ -5453,7 +5453,7 @@
         </is>
       </c>
       <c r="L61" s="17" t="n">
-        <v>253</v>
+        <v>417</v>
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
@@ -5526,7 +5526,7 @@
         </is>
       </c>
       <c r="L62" s="17" t="n">
-        <v>417</v>
+        <v>473</v>
       </c>
       <c r="M62" s="17" t="inlineStr">
         <is>
@@ -5599,7 +5599,7 @@
         </is>
       </c>
       <c r="L63" s="17" t="n">
-        <v>402</v>
+        <v>569</v>
       </c>
       <c r="M63" s="17" t="inlineStr">
         <is>
@@ -5672,7 +5672,7 @@
         </is>
       </c>
       <c r="L64" s="17" t="n">
-        <v>609</v>
+        <v>500</v>
       </c>
       <c r="M64" s="17" t="inlineStr">
         <is>
@@ -5745,7 +5745,7 @@
         </is>
       </c>
       <c r="L65" s="17" t="n">
-        <v>200</v>
+        <v>271</v>
       </c>
       <c r="M65" s="17" t="inlineStr">
         <is>
@@ -5818,7 +5818,7 @@
         </is>
       </c>
       <c r="L66" s="17" t="n">
-        <v>336</v>
+        <v>583</v>
       </c>
       <c r="M66" s="17" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         </is>
       </c>
       <c r="L67" s="17" t="n">
-        <v>202</v>
+        <v>277</v>
       </c>
       <c r="M67" s="17" t="inlineStr">
         <is>
@@ -5964,7 +5964,7 @@
         </is>
       </c>
       <c r="L68" s="17" t="n">
-        <v>397</v>
+        <v>557</v>
       </c>
       <c r="M68" s="17" t="inlineStr">
         <is>
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="L69" s="17" t="n">
-        <v>403</v>
+        <v>336</v>
       </c>
       <c r="M69" s="17" t="inlineStr">
         <is>
@@ -6110,7 +6110,7 @@
         </is>
       </c>
       <c r="L70" s="17" t="n">
-        <v>191</v>
+        <v>461</v>
       </c>
       <c r="M70" s="17" t="inlineStr">
         <is>
@@ -6183,7 +6183,7 @@
         </is>
       </c>
       <c r="L71" s="17" t="n">
-        <v>199</v>
+        <v>505</v>
       </c>
       <c r="M71" s="17" t="inlineStr">
         <is>
@@ -6256,7 +6256,7 @@
         </is>
       </c>
       <c r="L72" s="17" t="n">
-        <v>540</v>
+        <v>345</v>
       </c>
       <c r="M72" s="17" t="inlineStr">
         <is>
@@ -6329,7 +6329,7 @@
         </is>
       </c>
       <c r="L73" s="17" t="n">
-        <v>337</v>
+        <v>188</v>
       </c>
       <c r="M73" s="17" t="inlineStr">
         <is>
@@ -6402,7 +6402,7 @@
         </is>
       </c>
       <c r="L74" s="17" t="n">
-        <v>407</v>
+        <v>434</v>
       </c>
       <c r="M74" s="17" t="inlineStr">
         <is>
@@ -6475,7 +6475,7 @@
         </is>
       </c>
       <c r="L75" s="17" t="n">
-        <v>295</v>
+        <v>476</v>
       </c>
       <c r="M75" s="17" t="inlineStr">
         <is>
@@ -6548,7 +6548,7 @@
         </is>
       </c>
       <c r="L76" s="17" t="n">
-        <v>408</v>
+        <v>627</v>
       </c>
       <c r="M76" s="17" t="inlineStr">
         <is>
@@ -6621,7 +6621,7 @@
         </is>
       </c>
       <c r="L77" s="17" t="n">
-        <v>308</v>
+        <v>261</v>
       </c>
       <c r="M77" s="17" t="inlineStr">
         <is>
@@ -6694,7 +6694,7 @@
         </is>
       </c>
       <c r="L78" s="17" t="n">
-        <v>576</v>
+        <v>595</v>
       </c>
       <c r="M78" s="17" t="inlineStr">
         <is>
@@ -6767,7 +6767,7 @@
         </is>
       </c>
       <c r="L79" s="17" t="n">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="M79" s="17" t="inlineStr">
         <is>
@@ -6840,7 +6840,7 @@
         </is>
       </c>
       <c r="L80" s="17" t="n">
-        <v>350</v>
+        <v>396</v>
       </c>
       <c r="M80" s="17" t="inlineStr">
         <is>
@@ -6913,7 +6913,7 @@
         </is>
       </c>
       <c r="L81" s="17" t="n">
-        <v>604</v>
+        <v>300</v>
       </c>
       <c r="M81" s="17" t="inlineStr">
         <is>
@@ -6986,7 +6986,7 @@
         </is>
       </c>
       <c r="L82" s="17" t="n">
-        <v>236</v>
+        <v>278</v>
       </c>
       <c r="M82" s="17" t="inlineStr">
         <is>
@@ -7059,7 +7059,7 @@
         </is>
       </c>
       <c r="L83" s="17" t="n">
-        <v>245</v>
+        <v>500</v>
       </c>
       <c r="M83" s="17" t="inlineStr">
         <is>
@@ -7132,7 +7132,7 @@
         </is>
       </c>
       <c r="L84" s="17" t="n">
-        <v>550</v>
+        <v>512</v>
       </c>
       <c r="M84" s="17" t="inlineStr">
         <is>
@@ -7205,7 +7205,7 @@
         </is>
       </c>
       <c r="L85" s="17" t="n">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="M85" s="17" t="inlineStr">
         <is>
@@ -7278,7 +7278,7 @@
         </is>
       </c>
       <c r="L86" s="17" t="n">
-        <v>422</v>
+        <v>605</v>
       </c>
       <c r="M86" s="17" t="inlineStr">
         <is>
@@ -7351,7 +7351,7 @@
         </is>
       </c>
       <c r="L87" s="17" t="n">
-        <v>607</v>
+        <v>383</v>
       </c>
       <c r="M87" s="17" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         </is>
       </c>
       <c r="L88" s="17" t="n">
-        <v>503</v>
+        <v>204</v>
       </c>
       <c r="M88" s="17" t="inlineStr">
         <is>
@@ -7497,7 +7497,7 @@
         </is>
       </c>
       <c r="L89" s="17" t="n">
-        <v>609</v>
+        <v>368</v>
       </c>
       <c r="M89" s="17" t="inlineStr">
         <is>
@@ -7570,7 +7570,7 @@
         </is>
       </c>
       <c r="L90" s="17" t="n">
-        <v>346</v>
+        <v>614</v>
       </c>
       <c r="M90" s="17" t="inlineStr">
         <is>
@@ -7643,7 +7643,7 @@
         </is>
       </c>
       <c r="L91" s="17" t="n">
-        <v>394</v>
+        <v>280</v>
       </c>
       <c r="M91" s="17" t="inlineStr">
         <is>
@@ -7716,7 +7716,7 @@
         </is>
       </c>
       <c r="L92" s="17" t="n">
-        <v>516</v>
+        <v>183</v>
       </c>
       <c r="M92" s="17" t="inlineStr">
         <is>
@@ -7789,7 +7789,7 @@
         </is>
       </c>
       <c r="L93" s="17" t="n">
-        <v>296</v>
+        <v>382</v>
       </c>
       <c r="M93" s="17" t="inlineStr">
         <is>
@@ -7862,7 +7862,7 @@
         </is>
       </c>
       <c r="L94" s="17" t="n">
-        <v>193</v>
+        <v>240</v>
       </c>
       <c r="M94" s="17" t="inlineStr">
         <is>
@@ -7935,7 +7935,7 @@
         </is>
       </c>
       <c r="L95" s="17" t="n">
-        <v>636</v>
+        <v>291</v>
       </c>
       <c r="M95" s="17" t="inlineStr">
         <is>
@@ -8008,7 +8008,7 @@
         </is>
       </c>
       <c r="L96" s="17" t="n">
-        <v>628</v>
+        <v>218</v>
       </c>
       <c r="M96" s="17" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
         </is>
       </c>
       <c r="L97" s="17" t="n">
-        <v>188</v>
+        <v>221</v>
       </c>
       <c r="M97" s="17" t="inlineStr">
         <is>
@@ -8154,7 +8154,7 @@
         </is>
       </c>
       <c r="L98" s="17" t="n">
-        <v>498</v>
+        <v>363</v>
       </c>
       <c r="M98" s="17" t="inlineStr">
         <is>
@@ -8227,7 +8227,7 @@
         </is>
       </c>
       <c r="L99" s="17" t="n">
-        <v>351</v>
+        <v>519</v>
       </c>
       <c r="M99" s="17" t="inlineStr">
         <is>
@@ -8300,7 +8300,7 @@
         </is>
       </c>
       <c r="L100" s="17" t="n">
-        <v>613</v>
+        <v>412</v>
       </c>
       <c r="M100" s="17" t="inlineStr">
         <is>
@@ -8373,7 +8373,7 @@
         </is>
       </c>
       <c r="L101" s="17" t="n">
-        <v>251</v>
+        <v>623</v>
       </c>
       <c r="M101" s="17" t="inlineStr">
         <is>
@@ -8446,7 +8446,7 @@
         </is>
       </c>
       <c r="L102" s="17" t="n">
-        <v>298</v>
+        <v>252</v>
       </c>
       <c r="M102" s="17" t="inlineStr">
         <is>
@@ -8519,7 +8519,7 @@
         </is>
       </c>
       <c r="L103" s="17" t="n">
-        <v>527</v>
+        <v>509</v>
       </c>
       <c r="M103" s="17" t="inlineStr">
         <is>
@@ -8592,7 +8592,7 @@
         </is>
       </c>
       <c r="L104" s="17" t="n">
-        <v>290</v>
+        <v>624</v>
       </c>
       <c r="M104" s="17" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="L105" s="17" t="n">
-        <v>242</v>
+        <v>291</v>
       </c>
       <c r="M105" s="17" t="inlineStr">
         <is>
@@ -8738,7 +8738,7 @@
         </is>
       </c>
       <c r="L106" s="17" t="n">
-        <v>357</v>
+        <v>206</v>
       </c>
       <c r="M106" s="17" t="inlineStr">
         <is>
@@ -8811,7 +8811,7 @@
         </is>
       </c>
       <c r="L107" s="17" t="n">
-        <v>303</v>
+        <v>225</v>
       </c>
       <c r="M107" s="17" t="inlineStr">
         <is>
@@ -8884,7 +8884,7 @@
         </is>
       </c>
       <c r="L108" s="17" t="n">
-        <v>302</v>
+        <v>280</v>
       </c>
       <c r="M108" s="17" t="inlineStr">
         <is>
@@ -8957,7 +8957,7 @@
         </is>
       </c>
       <c r="L109" s="17" t="n">
-        <v>586</v>
+        <v>245</v>
       </c>
       <c r="M109" s="17" t="inlineStr">
         <is>
@@ -9030,7 +9030,7 @@
         </is>
       </c>
       <c r="L110" s="17" t="n">
-        <v>553</v>
+        <v>533</v>
       </c>
       <c r="M110" s="17" t="inlineStr">
         <is>
@@ -9103,7 +9103,7 @@
         </is>
       </c>
       <c r="L111" s="17" t="n">
-        <v>437</v>
+        <v>254</v>
       </c>
       <c r="M111" s="17" t="inlineStr">
         <is>
@@ -9176,7 +9176,7 @@
         </is>
       </c>
       <c r="L112" s="17" t="n">
-        <v>476</v>
+        <v>302</v>
       </c>
       <c r="M112" s="17" t="inlineStr">
         <is>
@@ -9249,7 +9249,7 @@
         </is>
       </c>
       <c r="L113" s="17" t="n">
-        <v>213</v>
+        <v>244</v>
       </c>
       <c r="M113" s="17" t="inlineStr">
         <is>
@@ -9322,7 +9322,7 @@
         </is>
       </c>
       <c r="L114" s="17" t="n">
-        <v>475</v>
+        <v>336</v>
       </c>
       <c r="M114" s="17" t="inlineStr">
         <is>
@@ -9395,7 +9395,7 @@
         </is>
       </c>
       <c r="L115" s="17" t="n">
-        <v>302</v>
+        <v>569</v>
       </c>
       <c r="M115" s="17" t="inlineStr">
         <is>
@@ -9468,7 +9468,7 @@
         </is>
       </c>
       <c r="L116" s="17" t="n">
-        <v>553</v>
+        <v>394</v>
       </c>
       <c r="M116" s="17" t="inlineStr">
         <is>
@@ -9541,7 +9541,7 @@
         </is>
       </c>
       <c r="L117" s="17" t="n">
-        <v>291</v>
+        <v>240</v>
       </c>
       <c r="M117" s="17" t="inlineStr">
         <is>
@@ -9614,7 +9614,7 @@
         </is>
       </c>
       <c r="L118" s="17" t="n">
-        <v>254</v>
+        <v>638</v>
       </c>
       <c r="M118" s="17" t="inlineStr">
         <is>
@@ -9687,7 +9687,7 @@
         </is>
       </c>
       <c r="L119" s="17" t="n">
-        <v>458</v>
+        <v>441</v>
       </c>
       <c r="M119" s="17" t="inlineStr">
         <is>
@@ -9760,7 +9760,7 @@
         </is>
       </c>
       <c r="L120" s="17" t="n">
-        <v>511</v>
+        <v>220</v>
       </c>
       <c r="M120" s="17" t="inlineStr">
         <is>
@@ -9833,7 +9833,7 @@
         </is>
       </c>
       <c r="L121" s="17" t="n">
-        <v>439</v>
+        <v>580</v>
       </c>
       <c r="M121" s="17" t="inlineStr">
         <is>
@@ -9906,7 +9906,7 @@
         </is>
       </c>
       <c r="L122" s="17" t="n">
-        <v>459</v>
+        <v>622</v>
       </c>
       <c r="M122" s="17" t="inlineStr">
         <is>
@@ -9979,7 +9979,7 @@
         </is>
       </c>
       <c r="L123" s="17" t="n">
-        <v>571</v>
+        <v>486</v>
       </c>
       <c r="M123" s="17" t="inlineStr">
         <is>
@@ -10052,7 +10052,7 @@
         </is>
       </c>
       <c r="L124" s="17" t="n">
-        <v>262</v>
+        <v>517</v>
       </c>
       <c r="M124" s="17" t="inlineStr">
         <is>
@@ -10125,7 +10125,7 @@
         </is>
       </c>
       <c r="L125" s="17" t="n">
-        <v>438</v>
+        <v>412</v>
       </c>
       <c r="M125" s="17" t="inlineStr">
         <is>
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="L126" s="17" t="n">
-        <v>191</v>
+        <v>218</v>
       </c>
       <c r="M126" s="17" t="inlineStr">
         <is>
@@ -10271,7 +10271,7 @@
         </is>
       </c>
       <c r="L127" s="17" t="n">
-        <v>598</v>
+        <v>314</v>
       </c>
       <c r="M127" s="17" t="inlineStr">
         <is>
@@ -10344,7 +10344,7 @@
         </is>
       </c>
       <c r="L128" s="17" t="n">
-        <v>438</v>
+        <v>300</v>
       </c>
       <c r="M128" s="17" t="inlineStr">
         <is>
@@ -10417,7 +10417,7 @@
         </is>
       </c>
       <c r="L129" s="17" t="n">
-        <v>579</v>
+        <v>445</v>
       </c>
       <c r="M129" s="17" t="inlineStr">
         <is>
@@ -10490,7 +10490,7 @@
         </is>
       </c>
       <c r="L130" s="17" t="n">
-        <v>279</v>
+        <v>548</v>
       </c>
       <c r="M130" s="17" t="inlineStr">
         <is>
@@ -10563,7 +10563,7 @@
         </is>
       </c>
       <c r="L131" s="17" t="n">
-        <v>551</v>
+        <v>644</v>
       </c>
       <c r="M131" s="17" t="inlineStr">
         <is>
@@ -10636,7 +10636,7 @@
         </is>
       </c>
       <c r="L132" s="17" t="n">
-        <v>269</v>
+        <v>360</v>
       </c>
       <c r="M132" s="17" t="inlineStr">
         <is>
@@ -10709,7 +10709,7 @@
         </is>
       </c>
       <c r="L133" s="17" t="n">
-        <v>424</v>
+        <v>319</v>
       </c>
       <c r="M133" s="17" t="inlineStr">
         <is>
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="L134" s="17" t="n">
-        <v>181</v>
+        <v>286</v>
       </c>
       <c r="M134" s="17" t="inlineStr">
         <is>
@@ -10855,7 +10855,7 @@
         </is>
       </c>
       <c r="L135" s="17" t="n">
-        <v>379</v>
+        <v>207</v>
       </c>
       <c r="M135" s="17" t="inlineStr">
         <is>
@@ -10928,7 +10928,7 @@
         </is>
       </c>
       <c r="L136" s="17" t="n">
-        <v>472</v>
+        <v>635</v>
       </c>
       <c r="M136" s="17" t="inlineStr">
         <is>
@@ -11001,7 +11001,7 @@
         </is>
       </c>
       <c r="L137" s="17" t="n">
-        <v>510</v>
+        <v>232</v>
       </c>
       <c r="M137" s="17" t="inlineStr">
         <is>
@@ -11074,7 +11074,7 @@
         </is>
       </c>
       <c r="L138" s="17" t="n">
-        <v>205</v>
+        <v>233</v>
       </c>
       <c r="M138" s="17" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
         </is>
       </c>
       <c r="L139" s="17" t="n">
-        <v>649</v>
+        <v>535</v>
       </c>
       <c r="M139" s="17" t="inlineStr">
         <is>
@@ -11220,7 +11220,7 @@
         </is>
       </c>
       <c r="L140" s="17" t="n">
-        <v>619</v>
+        <v>363</v>
       </c>
       <c r="M140" s="17" t="inlineStr">
         <is>
@@ -11293,7 +11293,7 @@
         </is>
       </c>
       <c r="L141" s="17" t="n">
-        <v>206</v>
+        <v>459</v>
       </c>
       <c r="M141" s="17" t="inlineStr">
         <is>
@@ -11366,7 +11366,7 @@
         </is>
       </c>
       <c r="L142" s="17" t="n">
-        <v>423</v>
+        <v>393</v>
       </c>
       <c r="M142" s="17" t="inlineStr">
         <is>
@@ -11439,7 +11439,7 @@
         </is>
       </c>
       <c r="L143" s="17" t="n">
-        <v>471</v>
+        <v>351</v>
       </c>
       <c r="M143" s="17" t="inlineStr">
         <is>
@@ -11512,7 +11512,7 @@
         </is>
       </c>
       <c r="L144" s="17" t="n">
-        <v>224</v>
+        <v>189</v>
       </c>
       <c r="M144" s="17" t="inlineStr">
         <is>
@@ -11585,7 +11585,7 @@
         </is>
       </c>
       <c r="L145" s="17" t="n">
-        <v>544</v>
+        <v>557</v>
       </c>
       <c r="M145" s="17" t="inlineStr">
         <is>
@@ -11658,7 +11658,7 @@
         </is>
       </c>
       <c r="L146" s="17" t="n">
-        <v>359</v>
+        <v>578</v>
       </c>
       <c r="M146" s="17" t="inlineStr">
         <is>
@@ -11731,7 +11731,7 @@
         </is>
       </c>
       <c r="L147" s="17" t="n">
-        <v>289</v>
+        <v>584</v>
       </c>
       <c r="M147" s="17" t="inlineStr">
         <is>
@@ -11804,7 +11804,7 @@
         </is>
       </c>
       <c r="L148" s="17" t="n">
-        <v>403</v>
+        <v>541</v>
       </c>
       <c r="M148" s="17" t="inlineStr">
         <is>
@@ -11877,7 +11877,7 @@
         </is>
       </c>
       <c r="L149" s="17" t="n">
-        <v>434</v>
+        <v>333</v>
       </c>
       <c r="M149" s="17" t="inlineStr">
         <is>
@@ -11950,7 +11950,7 @@
         </is>
       </c>
       <c r="L150" s="17" t="n">
-        <v>282</v>
+        <v>616</v>
       </c>
       <c r="M150" s="17" t="inlineStr">
         <is>
@@ -12023,7 +12023,7 @@
         </is>
       </c>
       <c r="L151" s="17" t="n">
-        <v>384</v>
+        <v>253</v>
       </c>
       <c r="M151" s="17" t="inlineStr">
         <is>
@@ -12096,7 +12096,7 @@
         </is>
       </c>
       <c r="L152" s="17" t="n">
-        <v>220</v>
+        <v>603</v>
       </c>
       <c r="M152" s="17" t="inlineStr">
         <is>
@@ -12169,7 +12169,7 @@
         </is>
       </c>
       <c r="L153" s="17" t="n">
-        <v>270</v>
+        <v>627</v>
       </c>
       <c r="M153" s="17" t="inlineStr">
         <is>
@@ -12242,7 +12242,7 @@
         </is>
       </c>
       <c r="L154" s="17" t="n">
-        <v>640</v>
+        <v>342</v>
       </c>
       <c r="M154" s="17" t="inlineStr">
         <is>
@@ -12315,7 +12315,7 @@
         </is>
       </c>
       <c r="L155" s="17" t="n">
-        <v>541</v>
+        <v>645</v>
       </c>
       <c r="M155" s="17" t="inlineStr">
         <is>
@@ -12388,7 +12388,7 @@
         </is>
       </c>
       <c r="L156" s="17" t="n">
-        <v>525</v>
+        <v>373</v>
       </c>
       <c r="M156" s="17" t="inlineStr">
         <is>
@@ -12461,7 +12461,7 @@
         </is>
       </c>
       <c r="L157" s="17" t="n">
-        <v>280</v>
+        <v>357</v>
       </c>
       <c r="M157" s="17" t="inlineStr">
         <is>
@@ -12534,7 +12534,7 @@
         </is>
       </c>
       <c r="L158" s="17" t="n">
-        <v>586</v>
+        <v>568</v>
       </c>
       <c r="M158" s="17" t="inlineStr">
         <is>
@@ -12607,7 +12607,7 @@
         </is>
       </c>
       <c r="L159" s="17" t="n">
-        <v>281</v>
+        <v>500</v>
       </c>
       <c r="M159" s="17" t="inlineStr">
         <is>
@@ -12680,7 +12680,7 @@
         </is>
       </c>
       <c r="L160" s="17" t="n">
-        <v>250</v>
+        <v>379</v>
       </c>
       <c r="M160" s="17" t="inlineStr">
         <is>
@@ -12753,7 +12753,7 @@
         </is>
       </c>
       <c r="L161" s="17" t="n">
-        <v>532</v>
+        <v>234</v>
       </c>
       <c r="M161" s="17" t="inlineStr">
         <is>
@@ -12826,7 +12826,7 @@
         </is>
       </c>
       <c r="L162" s="17" t="n">
-        <v>564</v>
+        <v>238</v>
       </c>
       <c r="M162" s="17" t="inlineStr">
         <is>
@@ -12899,7 +12899,7 @@
         </is>
       </c>
       <c r="L163" s="17" t="n">
-        <v>428</v>
+        <v>580</v>
       </c>
       <c r="M163" s="17" t="inlineStr">
         <is>
@@ -12972,7 +12972,7 @@
         </is>
       </c>
       <c r="L164" s="17" t="n">
-        <v>526</v>
+        <v>377</v>
       </c>
       <c r="M164" s="17" t="inlineStr">
         <is>
@@ -13045,7 +13045,7 @@
         </is>
       </c>
       <c r="L165" s="17" t="n">
-        <v>352</v>
+        <v>569</v>
       </c>
       <c r="M165" s="17" t="inlineStr">
         <is>
@@ -13118,7 +13118,7 @@
         </is>
       </c>
       <c r="L166" s="17" t="n">
-        <v>603</v>
+        <v>637</v>
       </c>
       <c r="M166" s="17" t="inlineStr">
         <is>
@@ -13191,7 +13191,7 @@
         </is>
       </c>
       <c r="L167" s="17" t="n">
-        <v>236</v>
+        <v>320</v>
       </c>
       <c r="M167" s="17" t="inlineStr">
         <is>
@@ -13264,7 +13264,7 @@
         </is>
       </c>
       <c r="L168" s="17" t="n">
-        <v>601</v>
+        <v>283</v>
       </c>
       <c r="M168" s="17" t="inlineStr">
         <is>
@@ -13337,7 +13337,7 @@
         </is>
       </c>
       <c r="L169" s="17" t="n">
-        <v>632</v>
+        <v>364</v>
       </c>
       <c r="M169" s="17" t="inlineStr">
         <is>
@@ -13410,7 +13410,7 @@
         </is>
       </c>
       <c r="L170" s="17" t="n">
-        <v>181</v>
+        <v>349</v>
       </c>
       <c r="M170" s="17" t="inlineStr">
         <is>
@@ -13483,7 +13483,7 @@
         </is>
       </c>
       <c r="L171" s="17" t="n">
-        <v>639</v>
+        <v>235</v>
       </c>
       <c r="M171" s="17" t="inlineStr">
         <is>
@@ -13556,7 +13556,7 @@
         </is>
       </c>
       <c r="L172" s="17" t="n">
-        <v>277</v>
+        <v>595</v>
       </c>
       <c r="M172" s="17" t="inlineStr">
         <is>
@@ -13629,7 +13629,7 @@
         </is>
       </c>
       <c r="L173" s="17" t="n">
-        <v>255</v>
+        <v>277</v>
       </c>
       <c r="M173" s="17" t="inlineStr">
         <is>
@@ -13702,7 +13702,7 @@
         </is>
       </c>
       <c r="L174" s="17" t="n">
-        <v>570</v>
+        <v>339</v>
       </c>
       <c r="M174" s="17" t="inlineStr">
         <is>
@@ -13775,7 +13775,7 @@
         </is>
       </c>
       <c r="L175" s="17" t="n">
-        <v>455</v>
+        <v>383</v>
       </c>
       <c r="M175" s="17" t="inlineStr">
         <is>
@@ -13848,7 +13848,7 @@
         </is>
       </c>
       <c r="L176" s="17" t="n">
-        <v>381</v>
+        <v>276</v>
       </c>
       <c r="M176" s="17" t="inlineStr">
         <is>
@@ -13921,7 +13921,7 @@
         </is>
       </c>
       <c r="L177" s="17" t="n">
-        <v>359</v>
+        <v>227</v>
       </c>
       <c r="M177" s="17" t="inlineStr">
         <is>
@@ -13994,7 +13994,7 @@
         </is>
       </c>
       <c r="L178" s="17" t="n">
-        <v>259</v>
+        <v>435</v>
       </c>
       <c r="M178" s="17" t="inlineStr">
         <is>
@@ -14067,7 +14067,7 @@
         </is>
       </c>
       <c r="L179" s="17" t="n">
-        <v>223</v>
+        <v>369</v>
       </c>
       <c r="M179" s="17" t="inlineStr">
         <is>
@@ -14140,7 +14140,7 @@
         </is>
       </c>
       <c r="L180" s="17" t="n">
-        <v>289</v>
+        <v>431</v>
       </c>
       <c r="M180" s="17" t="inlineStr">
         <is>
@@ -14213,7 +14213,7 @@
         </is>
       </c>
       <c r="L181" s="17" t="n">
-        <v>565</v>
+        <v>347</v>
       </c>
       <c r="M181" s="17" t="inlineStr">
         <is>
@@ -14286,7 +14286,7 @@
         </is>
       </c>
       <c r="L182" s="17" t="n">
-        <v>582</v>
+        <v>228</v>
       </c>
       <c r="M182" s="17" t="inlineStr">
         <is>
@@ -14359,7 +14359,7 @@
         </is>
       </c>
       <c r="L183" s="17" t="n">
-        <v>364</v>
+        <v>278</v>
       </c>
       <c r="M183" s="17" t="inlineStr">
         <is>
@@ -14432,7 +14432,7 @@
         </is>
       </c>
       <c r="L184" s="17" t="n">
-        <v>638</v>
+        <v>432</v>
       </c>
       <c r="M184" s="17" t="inlineStr">
         <is>
@@ -14505,7 +14505,7 @@
         </is>
       </c>
       <c r="L185" s="17" t="n">
-        <v>459</v>
+        <v>641</v>
       </c>
       <c r="M185" s="17" t="inlineStr">
         <is>
@@ -14578,7 +14578,7 @@
         </is>
       </c>
       <c r="L186" s="17" t="n">
-        <v>430</v>
+        <v>391</v>
       </c>
       <c r="M186" s="17" t="inlineStr">
         <is>
@@ -14651,7 +14651,7 @@
         </is>
       </c>
       <c r="L187" s="17" t="n">
-        <v>603</v>
+        <v>219</v>
       </c>
       <c r="M187" s="17" t="inlineStr">
         <is>
@@ -14724,7 +14724,7 @@
         </is>
       </c>
       <c r="L188" s="17" t="n">
-        <v>321</v>
+        <v>482</v>
       </c>
       <c r="M188" s="17" t="inlineStr">
         <is>
@@ -14797,7 +14797,7 @@
         </is>
       </c>
       <c r="L189" s="17" t="n">
-        <v>287</v>
+        <v>415</v>
       </c>
       <c r="M189" s="17" t="inlineStr">
         <is>
@@ -14870,7 +14870,7 @@
         </is>
       </c>
       <c r="L190" s="17" t="n">
-        <v>325</v>
+        <v>196</v>
       </c>
       <c r="M190" s="17" t="inlineStr">
         <is>
@@ -14943,7 +14943,7 @@
         </is>
       </c>
       <c r="L191" s="17" t="n">
-        <v>549</v>
+        <v>259</v>
       </c>
       <c r="M191" s="17" t="inlineStr">
         <is>
@@ -15016,7 +15016,7 @@
         </is>
       </c>
       <c r="L192" s="17" t="n">
-        <v>596</v>
+        <v>201</v>
       </c>
       <c r="M192" s="17" t="inlineStr">
         <is>
@@ -15089,7 +15089,7 @@
         </is>
       </c>
       <c r="L193" s="17" t="n">
-        <v>622</v>
+        <v>372</v>
       </c>
       <c r="M193" s="17" t="inlineStr">
         <is>
@@ -15162,7 +15162,7 @@
         </is>
       </c>
       <c r="L194" s="17" t="n">
-        <v>414</v>
+        <v>439</v>
       </c>
       <c r="M194" s="17" t="inlineStr">
         <is>
@@ -15235,7 +15235,7 @@
         </is>
       </c>
       <c r="L195" s="17" t="n">
-        <v>234</v>
+        <v>647</v>
       </c>
       <c r="M195" s="17" t="inlineStr">
         <is>
@@ -15308,7 +15308,7 @@
         </is>
       </c>
       <c r="L196" s="17" t="n">
-        <v>309</v>
+        <v>494</v>
       </c>
       <c r="M196" s="17" t="inlineStr">
         <is>
@@ -15381,7 +15381,7 @@
         </is>
       </c>
       <c r="L197" s="17" t="n">
-        <v>224</v>
+        <v>379</v>
       </c>
       <c r="M197" s="17" t="inlineStr">
         <is>
@@ -15454,7 +15454,7 @@
         </is>
       </c>
       <c r="L198" s="17" t="n">
-        <v>505</v>
+        <v>381</v>
       </c>
       <c r="M198" s="17" t="inlineStr">
         <is>
@@ -15527,7 +15527,7 @@
         </is>
       </c>
       <c r="L199" s="17" t="n">
-        <v>436</v>
+        <v>598</v>
       </c>
       <c r="M199" s="17" t="inlineStr">
         <is>
@@ -15600,7 +15600,7 @@
         </is>
       </c>
       <c r="L200" s="17" t="n">
-        <v>262</v>
+        <v>639</v>
       </c>
       <c r="M200" s="17" t="inlineStr">
         <is>
@@ -15673,7 +15673,7 @@
         </is>
       </c>
       <c r="L201" s="17" t="n">
-        <v>495</v>
+        <v>213</v>
       </c>
       <c r="M201" s="17" t="inlineStr">
         <is>
@@ -15746,7 +15746,7 @@
         </is>
       </c>
       <c r="L202" s="17" t="n">
-        <v>508</v>
+        <v>648</v>
       </c>
       <c r="M202" s="17" t="inlineStr">
         <is>
@@ -15819,7 +15819,7 @@
         </is>
       </c>
       <c r="L203" s="17" t="n">
-        <v>307</v>
+        <v>250</v>
       </c>
       <c r="M203" s="17" t="inlineStr">
         <is>
@@ -15892,7 +15892,7 @@
         </is>
       </c>
       <c r="L204" s="17" t="n">
-        <v>282</v>
+        <v>236</v>
       </c>
       <c r="M204" s="17" t="inlineStr">
         <is>
@@ -15965,7 +15965,7 @@
         </is>
       </c>
       <c r="L205" s="17" t="n">
-        <v>335</v>
+        <v>305</v>
       </c>
       <c r="M205" s="17" t="inlineStr">
         <is>
@@ -16038,7 +16038,7 @@
         </is>
       </c>
       <c r="L206" s="17" t="n">
-        <v>618</v>
+        <v>456</v>
       </c>
       <c r="M206" s="17" t="inlineStr">
         <is>
@@ -16111,7 +16111,7 @@
         </is>
       </c>
       <c r="L207" s="17" t="n">
-        <v>566</v>
+        <v>184</v>
       </c>
       <c r="M207" s="17" t="inlineStr">
         <is>
@@ -16184,7 +16184,7 @@
         </is>
       </c>
       <c r="L208" s="17" t="n">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="M208" s="17" t="inlineStr">
         <is>
@@ -16257,7 +16257,7 @@
         </is>
       </c>
       <c r="L209" s="17" t="n">
-        <v>410</v>
+        <v>205</v>
       </c>
       <c r="M209" s="17" t="inlineStr">
         <is>
@@ -16330,7 +16330,7 @@
         </is>
       </c>
       <c r="L210" s="17" t="n">
-        <v>604</v>
+        <v>339</v>
       </c>
       <c r="M210" s="17" t="inlineStr">
         <is>
@@ -16403,7 +16403,7 @@
         </is>
       </c>
       <c r="L211" s="17" t="n">
-        <v>431</v>
+        <v>300</v>
       </c>
       <c r="M211" s="17" t="inlineStr">
         <is>
@@ -16476,7 +16476,7 @@
         </is>
       </c>
       <c r="L212" s="17" t="n">
-        <v>559</v>
+        <v>392</v>
       </c>
       <c r="M212" s="17" t="inlineStr">
         <is>
@@ -16549,7 +16549,7 @@
         </is>
       </c>
       <c r="L213" s="17" t="n">
-        <v>343</v>
+        <v>531</v>
       </c>
       <c r="M213" s="17" t="inlineStr">
         <is>
@@ -16622,7 +16622,7 @@
         </is>
       </c>
       <c r="L214" s="17" t="n">
-        <v>407</v>
+        <v>488</v>
       </c>
       <c r="M214" s="17" t="inlineStr">
         <is>
@@ -16695,7 +16695,7 @@
         </is>
       </c>
       <c r="L215" s="17" t="n">
-        <v>245</v>
+        <v>582</v>
       </c>
       <c r="M215" s="17" t="inlineStr">
         <is>
@@ -16768,7 +16768,7 @@
         </is>
       </c>
       <c r="L216" s="17" t="n">
-        <v>585</v>
+        <v>454</v>
       </c>
       <c r="M216" s="17" t="inlineStr">
         <is>
@@ -16841,7 +16841,7 @@
         </is>
       </c>
       <c r="L217" s="17" t="n">
-        <v>292</v>
+        <v>228</v>
       </c>
       <c r="M217" s="17" t="inlineStr">
         <is>
@@ -16914,7 +16914,7 @@
         </is>
       </c>
       <c r="L218" s="17" t="n">
-        <v>419</v>
+        <v>635</v>
       </c>
       <c r="M218" s="17" t="inlineStr">
         <is>
@@ -16987,7 +16987,7 @@
         </is>
       </c>
       <c r="L219" s="17" t="n">
-        <v>363</v>
+        <v>490</v>
       </c>
       <c r="M219" s="17" t="inlineStr">
         <is>
@@ -17060,7 +17060,7 @@
         </is>
       </c>
       <c r="L220" s="17" t="n">
-        <v>588</v>
+        <v>358</v>
       </c>
       <c r="M220" s="17" t="inlineStr">
         <is>
@@ -17133,7 +17133,7 @@
         </is>
       </c>
       <c r="L221" s="17" t="n">
-        <v>441</v>
+        <v>451</v>
       </c>
       <c r="M221" s="17" t="inlineStr">
         <is>
@@ -17206,7 +17206,7 @@
         </is>
       </c>
       <c r="L222" s="17" t="n">
-        <v>460</v>
+        <v>387</v>
       </c>
       <c r="M222" s="17" t="inlineStr">
         <is>
@@ -17279,7 +17279,7 @@
         </is>
       </c>
       <c r="L223" s="17" t="n">
-        <v>591</v>
+        <v>284</v>
       </c>
       <c r="M223" s="17" t="inlineStr">
         <is>
@@ -17352,7 +17352,7 @@
         </is>
       </c>
       <c r="L224" s="17" t="n">
-        <v>203</v>
+        <v>640</v>
       </c>
       <c r="M224" s="17" t="inlineStr">
         <is>
@@ -17425,7 +17425,7 @@
         </is>
       </c>
       <c r="L225" s="17" t="n">
-        <v>433</v>
+        <v>551</v>
       </c>
       <c r="M225" s="17" t="inlineStr">
         <is>
@@ -17498,7 +17498,7 @@
         </is>
       </c>
       <c r="L226" s="17" t="n">
-        <v>319</v>
+        <v>356</v>
       </c>
       <c r="M226" s="17" t="inlineStr">
         <is>
@@ -17571,7 +17571,7 @@
         </is>
       </c>
       <c r="L227" s="17" t="n">
-        <v>227</v>
+        <v>507</v>
       </c>
       <c r="M227" s="17" t="inlineStr">
         <is>
@@ -17644,7 +17644,7 @@
         </is>
       </c>
       <c r="L228" s="17" t="n">
-        <v>618</v>
+        <v>633</v>
       </c>
       <c r="M228" s="17" t="inlineStr">
         <is>
@@ -17717,7 +17717,7 @@
         </is>
       </c>
       <c r="L229" s="17" t="n">
-        <v>608</v>
+        <v>485</v>
       </c>
       <c r="M229" s="17" t="inlineStr">
         <is>
@@ -17790,7 +17790,7 @@
         </is>
       </c>
       <c r="L230" s="17" t="n">
-        <v>228</v>
+        <v>181</v>
       </c>
       <c r="M230" s="17" t="inlineStr">
         <is>
@@ -17863,7 +17863,7 @@
         </is>
       </c>
       <c r="L231" s="17" t="n">
-        <v>222</v>
+        <v>476</v>
       </c>
       <c r="M231" s="17" t="inlineStr">
         <is>
@@ -17936,7 +17936,7 @@
         </is>
       </c>
       <c r="L232" s="17" t="n">
-        <v>508</v>
+        <v>240</v>
       </c>
       <c r="M232" s="17" t="inlineStr">
         <is>
@@ -18009,7 +18009,7 @@
         </is>
       </c>
       <c r="L233" s="17" t="n">
-        <v>310</v>
+        <v>625</v>
       </c>
       <c r="M233" s="17" t="inlineStr">
         <is>
@@ -18082,7 +18082,7 @@
         </is>
       </c>
       <c r="L234" s="17" t="n">
-        <v>223</v>
+        <v>589</v>
       </c>
       <c r="M234" s="17" t="inlineStr">
         <is>
@@ -18155,7 +18155,7 @@
         </is>
       </c>
       <c r="L235" s="17" t="n">
-        <v>182</v>
+        <v>414</v>
       </c>
       <c r="M235" s="17" t="inlineStr">
         <is>
@@ -18228,7 +18228,7 @@
         </is>
       </c>
       <c r="L236" s="17" t="n">
-        <v>370</v>
+        <v>261</v>
       </c>
       <c r="M236" s="17" t="inlineStr">
         <is>
@@ -18301,7 +18301,7 @@
         </is>
       </c>
       <c r="L237" s="17" t="n">
-        <v>232</v>
+        <v>190</v>
       </c>
       <c r="M237" s="17" t="inlineStr">
         <is>
@@ -18374,7 +18374,7 @@
         </is>
       </c>
       <c r="L238" s="17" t="n">
-        <v>355</v>
+        <v>413</v>
       </c>
       <c r="M238" s="17" t="inlineStr">
         <is>
@@ -18447,7 +18447,7 @@
         </is>
       </c>
       <c r="L239" s="17" t="n">
-        <v>521</v>
+        <v>238</v>
       </c>
       <c r="M239" s="17" t="inlineStr">
         <is>
@@ -18520,7 +18520,7 @@
         </is>
       </c>
       <c r="L240" s="17" t="n">
-        <v>596</v>
+        <v>265</v>
       </c>
       <c r="M240" s="17" t="inlineStr">
         <is>
@@ -18593,7 +18593,7 @@
         </is>
       </c>
       <c r="L241" s="17" t="n">
-        <v>393</v>
+        <v>477</v>
       </c>
       <c r="M241" s="17" t="inlineStr">
         <is>
@@ -18666,7 +18666,7 @@
         </is>
       </c>
       <c r="L242" s="17" t="n">
-        <v>494</v>
+        <v>443</v>
       </c>
       <c r="M242" s="17" t="inlineStr">
         <is>
@@ -18739,7 +18739,7 @@
         </is>
       </c>
       <c r="L243" s="17" t="n">
-        <v>625</v>
+        <v>294</v>
       </c>
       <c r="M243" s="17" t="inlineStr">
         <is>
@@ -18812,7 +18812,7 @@
         </is>
       </c>
       <c r="L244" s="17" t="n">
-        <v>462</v>
+        <v>518</v>
       </c>
       <c r="M244" s="17" t="inlineStr">
         <is>
@@ -18885,7 +18885,7 @@
         </is>
       </c>
       <c r="L245" s="17" t="n">
-        <v>394</v>
+        <v>644</v>
       </c>
       <c r="M245" s="17" t="inlineStr">
         <is>
@@ -18958,7 +18958,7 @@
         </is>
       </c>
       <c r="L246" s="17" t="n">
-        <v>364</v>
+        <v>623</v>
       </c>
       <c r="M246" s="17" t="inlineStr">
         <is>
@@ -19031,7 +19031,7 @@
         </is>
       </c>
       <c r="L247" s="17" t="n">
-        <v>291</v>
+        <v>617</v>
       </c>
       <c r="M247" s="17" t="inlineStr">
         <is>
@@ -19104,7 +19104,7 @@
         </is>
       </c>
       <c r="L248" s="17" t="n">
-        <v>296</v>
+        <v>355</v>
       </c>
       <c r="M248" s="17" t="inlineStr">
         <is>
@@ -19177,7 +19177,7 @@
         </is>
       </c>
       <c r="L249" s="17" t="n">
-        <v>223</v>
+        <v>638</v>
       </c>
       <c r="M249" s="17" t="inlineStr">
         <is>
@@ -19250,7 +19250,7 @@
         </is>
       </c>
       <c r="L250" s="17" t="n">
-        <v>453</v>
+        <v>485</v>
       </c>
       <c r="M250" s="17" t="inlineStr">
         <is>
@@ -19323,7 +19323,7 @@
         </is>
       </c>
       <c r="L251" s="17" t="n">
-        <v>502</v>
+        <v>241</v>
       </c>
       <c r="M251" s="17" t="inlineStr">
         <is>
@@ -19396,7 +19396,7 @@
         </is>
       </c>
       <c r="L252" s="17" t="n">
-        <v>377</v>
+        <v>336</v>
       </c>
       <c r="M252" s="17" t="inlineStr">
         <is>
@@ -19469,7 +19469,7 @@
         </is>
       </c>
       <c r="L253" s="17" t="n">
-        <v>431</v>
+        <v>198</v>
       </c>
       <c r="M253" s="17" t="inlineStr">
         <is>
@@ -19542,7 +19542,7 @@
         </is>
       </c>
       <c r="L254" s="17" t="n">
-        <v>532</v>
+        <v>617</v>
       </c>
       <c r="M254" s="17" t="inlineStr">
         <is>
@@ -19615,7 +19615,7 @@
         </is>
       </c>
       <c r="L255" s="17" t="n">
-        <v>278</v>
+        <v>416</v>
       </c>
       <c r="M255" s="17" t="inlineStr">
         <is>
@@ -19688,7 +19688,7 @@
         </is>
       </c>
       <c r="L256" s="17" t="n">
-        <v>241</v>
+        <v>216</v>
       </c>
       <c r="M256" s="17" t="inlineStr">
         <is>
@@ -19761,7 +19761,7 @@
         </is>
       </c>
       <c r="L257" s="17" t="n">
-        <v>545</v>
+        <v>488</v>
       </c>
       <c r="M257" s="17" t="inlineStr">
         <is>
@@ -19834,7 +19834,7 @@
         </is>
       </c>
       <c r="L258" s="17" t="n">
-        <v>338</v>
+        <v>530</v>
       </c>
       <c r="M258" s="17" t="inlineStr">
         <is>
@@ -19907,7 +19907,7 @@
         </is>
       </c>
       <c r="L259" s="17" t="n">
-        <v>207</v>
+        <v>518</v>
       </c>
       <c r="M259" s="17" t="inlineStr">
         <is>
@@ -19980,7 +19980,7 @@
         </is>
       </c>
       <c r="L260" s="17" t="n">
-        <v>538</v>
+        <v>588</v>
       </c>
       <c r="M260" s="17" t="inlineStr">
         <is>
@@ -20053,7 +20053,7 @@
         </is>
       </c>
       <c r="L261" s="17" t="n">
-        <v>601</v>
+        <v>225</v>
       </c>
       <c r="M261" s="17" t="inlineStr">
         <is>
@@ -20126,7 +20126,7 @@
         </is>
       </c>
       <c r="L262" s="17" t="n">
-        <v>287</v>
+        <v>384</v>
       </c>
       <c r="M262" s="17" t="inlineStr">
         <is>
@@ -20199,7 +20199,7 @@
         </is>
       </c>
       <c r="L263" s="17" t="n">
-        <v>242</v>
+        <v>463</v>
       </c>
       <c r="M263" s="17" t="inlineStr">
         <is>
@@ -20272,7 +20272,7 @@
         </is>
       </c>
       <c r="L264" s="17" t="n">
-        <v>474</v>
+        <v>310</v>
       </c>
       <c r="M264" s="17" t="inlineStr">
         <is>
@@ -20345,7 +20345,7 @@
         </is>
       </c>
       <c r="L265" s="17" t="n">
-        <v>495</v>
+        <v>483</v>
       </c>
       <c r="M265" s="17" t="inlineStr">
         <is>
@@ -20418,7 +20418,7 @@
         </is>
       </c>
       <c r="L266" s="17" t="n">
-        <v>368</v>
+        <v>445</v>
       </c>
       <c r="M266" s="17" t="inlineStr">
         <is>
@@ -20491,7 +20491,7 @@
         </is>
       </c>
       <c r="L267" s="17" t="n">
-        <v>507</v>
+        <v>214</v>
       </c>
       <c r="M267" s="17" t="inlineStr">
         <is>
@@ -20564,7 +20564,7 @@
         </is>
       </c>
       <c r="L268" s="17" t="n">
-        <v>433</v>
+        <v>240</v>
       </c>
       <c r="M268" s="17" t="inlineStr">
         <is>
@@ -20637,7 +20637,7 @@
         </is>
       </c>
       <c r="L269" s="17" t="n">
-        <v>583</v>
+        <v>523</v>
       </c>
       <c r="M269" s="17" t="inlineStr">
         <is>
@@ -20710,7 +20710,7 @@
         </is>
       </c>
       <c r="L270" s="17" t="n">
-        <v>188</v>
+        <v>469</v>
       </c>
       <c r="M270" s="17" t="inlineStr">
         <is>
@@ -20783,7 +20783,7 @@
         </is>
       </c>
       <c r="L271" s="17" t="n">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="M271" s="17" t="inlineStr">
         <is>
@@ -20856,7 +20856,7 @@
         </is>
       </c>
       <c r="L272" s="17" t="n">
-        <v>301</v>
+        <v>414</v>
       </c>
       <c r="M272" s="17" t="inlineStr">
         <is>
@@ -20929,7 +20929,7 @@
         </is>
       </c>
       <c r="L273" s="17" t="n">
-        <v>605</v>
+        <v>219</v>
       </c>
       <c r="M273" s="17" t="inlineStr">
         <is>
@@ -21002,7 +21002,7 @@
         </is>
       </c>
       <c r="L274" s="17" t="n">
-        <v>233</v>
+        <v>640</v>
       </c>
       <c r="M274" s="17" t="inlineStr">
         <is>
@@ -21075,7 +21075,7 @@
         </is>
       </c>
       <c r="L275" s="17" t="n">
-        <v>592</v>
+        <v>498</v>
       </c>
       <c r="M275" s="17" t="inlineStr">
         <is>
@@ -21148,7 +21148,7 @@
         </is>
       </c>
       <c r="L276" s="17" t="n">
-        <v>637</v>
+        <v>546</v>
       </c>
       <c r="M276" s="17" t="inlineStr">
         <is>
@@ -21221,7 +21221,7 @@
         </is>
       </c>
       <c r="L277" s="17" t="n">
-        <v>444</v>
+        <v>369</v>
       </c>
       <c r="M277" s="17" t="inlineStr">
         <is>
@@ -21294,7 +21294,7 @@
         </is>
       </c>
       <c r="L278" s="17" t="n">
-        <v>546</v>
+        <v>471</v>
       </c>
       <c r="M278" s="17" t="inlineStr">
         <is>
@@ -21367,7 +21367,7 @@
         </is>
       </c>
       <c r="L279" s="17" t="n">
-        <v>468</v>
+        <v>423</v>
       </c>
       <c r="M279" s="17" t="inlineStr">
         <is>
@@ -21440,7 +21440,7 @@
         </is>
       </c>
       <c r="L280" s="17" t="n">
-        <v>588</v>
+        <v>553</v>
       </c>
       <c r="M280" s="17" t="inlineStr">
         <is>
@@ -21513,7 +21513,7 @@
         </is>
       </c>
       <c r="L281" s="17" t="n">
-        <v>192</v>
+        <v>268</v>
       </c>
       <c r="M281" s="17" t="inlineStr">
         <is>
@@ -21586,7 +21586,7 @@
         </is>
       </c>
       <c r="L282" s="17" t="n">
-        <v>601</v>
+        <v>434</v>
       </c>
       <c r="M282" s="17" t="inlineStr">
         <is>
@@ -21659,7 +21659,7 @@
         </is>
       </c>
       <c r="L283" s="17" t="n">
-        <v>453</v>
+        <v>221</v>
       </c>
       <c r="M283" s="17" t="inlineStr">
         <is>
@@ -21732,7 +21732,7 @@
         </is>
       </c>
       <c r="L284" s="17" t="n">
-        <v>339</v>
+        <v>439</v>
       </c>
       <c r="M284" s="17" t="inlineStr">
         <is>
@@ -21805,7 +21805,7 @@
         </is>
       </c>
       <c r="L285" s="17" t="n">
-        <v>476</v>
+        <v>294</v>
       </c>
       <c r="M285" s="17" t="inlineStr">
         <is>
@@ -21878,7 +21878,7 @@
         </is>
       </c>
       <c r="L286" s="17" t="n">
-        <v>280</v>
+        <v>544</v>
       </c>
       <c r="M286" s="17" t="inlineStr">
         <is>
@@ -21951,7 +21951,7 @@
         </is>
       </c>
       <c r="L287" s="17" t="n">
-        <v>231</v>
+        <v>498</v>
       </c>
       <c r="M287" s="17" t="inlineStr">
         <is>
@@ -22024,7 +22024,7 @@
         </is>
       </c>
       <c r="L288" s="17" t="n">
-        <v>435</v>
+        <v>547</v>
       </c>
       <c r="M288" s="17" t="inlineStr">
         <is>
@@ -22097,7 +22097,7 @@
         </is>
       </c>
       <c r="L289" s="17" t="n">
-        <v>648</v>
+        <v>581</v>
       </c>
       <c r="M289" s="17" t="inlineStr">
         <is>
@@ -22170,7 +22170,7 @@
         </is>
       </c>
       <c r="L290" s="17" t="n">
-        <v>477</v>
+        <v>643</v>
       </c>
       <c r="M290" s="17" t="inlineStr">
         <is>
@@ -22243,7 +22243,7 @@
         </is>
       </c>
       <c r="L291" s="17" t="n">
-        <v>645</v>
+        <v>202</v>
       </c>
       <c r="M291" s="17" t="inlineStr">
         <is>
@@ -22316,7 +22316,7 @@
         </is>
       </c>
       <c r="L292" s="17" t="n">
-        <v>563</v>
+        <v>183</v>
       </c>
       <c r="M292" s="17" t="inlineStr">
         <is>
@@ -22389,7 +22389,7 @@
         </is>
       </c>
       <c r="L293" s="17" t="n">
-        <v>297</v>
+        <v>549</v>
       </c>
       <c r="M293" s="17" t="inlineStr">
         <is>
@@ -22462,7 +22462,7 @@
         </is>
       </c>
       <c r="L294" s="17" t="n">
-        <v>427</v>
+        <v>483</v>
       </c>
       <c r="M294" s="17" t="inlineStr">
         <is>
@@ -22535,7 +22535,7 @@
         </is>
       </c>
       <c r="L295" s="17" t="n">
-        <v>370</v>
+        <v>529</v>
       </c>
       <c r="M295" s="17" t="inlineStr">
         <is>
@@ -22608,7 +22608,7 @@
         </is>
       </c>
       <c r="L296" s="17" t="n">
-        <v>320</v>
+        <v>391</v>
       </c>
       <c r="M296" s="17" t="inlineStr">
         <is>
@@ -22681,7 +22681,7 @@
         </is>
       </c>
       <c r="L297" s="17" t="n">
-        <v>634</v>
+        <v>581</v>
       </c>
       <c r="M297" s="17" t="inlineStr">
         <is>
@@ -22754,7 +22754,7 @@
         </is>
       </c>
       <c r="L298" s="17" t="n">
-        <v>280</v>
+        <v>373</v>
       </c>
       <c r="M298" s="17" t="inlineStr">
         <is>
@@ -22827,7 +22827,7 @@
         </is>
       </c>
       <c r="L299" s="17" t="n">
-        <v>189</v>
+        <v>592</v>
       </c>
       <c r="M299" s="17" t="inlineStr">
         <is>
@@ -22900,7 +22900,7 @@
         </is>
       </c>
       <c r="L300" s="17" t="n">
-        <v>416</v>
+        <v>309</v>
       </c>
       <c r="M300" s="17" t="inlineStr">
         <is>
@@ -22973,7 +22973,7 @@
         </is>
       </c>
       <c r="L301" s="17" t="n">
-        <v>274</v>
+        <v>438</v>
       </c>
       <c r="M301" s="17" t="inlineStr">
         <is>
@@ -23046,7 +23046,7 @@
         </is>
       </c>
       <c r="L302" s="17" t="n">
-        <v>425</v>
+        <v>416</v>
       </c>
       <c r="M302" s="17" t="inlineStr">
         <is>
@@ -23119,7 +23119,7 @@
         </is>
       </c>
       <c r="L303" s="17" t="n">
-        <v>223</v>
+        <v>487</v>
       </c>
       <c r="M303" s="17" t="inlineStr">
         <is>
@@ -23192,7 +23192,7 @@
         </is>
       </c>
       <c r="L304" s="17" t="n">
-        <v>224</v>
+        <v>557</v>
       </c>
       <c r="M304" s="17" t="inlineStr">
         <is>
@@ -23265,7 +23265,7 @@
         </is>
       </c>
       <c r="L305" s="17" t="n">
-        <v>319</v>
+        <v>591</v>
       </c>
       <c r="M305" s="17" t="inlineStr">
         <is>
@@ -23338,7 +23338,7 @@
         </is>
       </c>
       <c r="L306" s="17" t="n">
-        <v>299</v>
+        <v>252</v>
       </c>
       <c r="M306" s="17" t="inlineStr">
         <is>
@@ -23411,7 +23411,7 @@
         </is>
       </c>
       <c r="L307" s="17" t="n">
-        <v>557</v>
+        <v>286</v>
       </c>
       <c r="M307" s="17" t="inlineStr">
         <is>
@@ -23484,7 +23484,7 @@
         </is>
       </c>
       <c r="L308" s="17" t="n">
-        <v>358</v>
+        <v>602</v>
       </c>
       <c r="M308" s="17" t="inlineStr">
         <is>
@@ -23557,7 +23557,7 @@
         </is>
       </c>
       <c r="L309" s="17" t="n">
-        <v>439</v>
+        <v>257</v>
       </c>
       <c r="M309" s="17" t="inlineStr">
         <is>
@@ -23630,7 +23630,7 @@
         </is>
       </c>
       <c r="L310" s="17" t="n">
-        <v>555</v>
+        <v>272</v>
       </c>
       <c r="M310" s="17" t="inlineStr">
         <is>
@@ -23703,7 +23703,7 @@
         </is>
       </c>
       <c r="L311" s="17" t="n">
-        <v>252</v>
+        <v>199</v>
       </c>
       <c r="M311" s="17" t="inlineStr">
         <is>
@@ -23776,7 +23776,7 @@
         </is>
       </c>
       <c r="L312" s="17" t="n">
-        <v>249</v>
+        <v>594</v>
       </c>
       <c r="M312" s="17" t="inlineStr">
         <is>
@@ -23849,7 +23849,7 @@
         </is>
       </c>
       <c r="L313" s="17" t="n">
-        <v>282</v>
+        <v>369</v>
       </c>
       <c r="M313" s="17" t="inlineStr">
         <is>
@@ -23922,7 +23922,7 @@
         </is>
       </c>
       <c r="L314" s="17" t="n">
-        <v>428</v>
+        <v>333</v>
       </c>
       <c r="M314" s="17" t="inlineStr">
         <is>
@@ -23995,7 +23995,7 @@
         </is>
       </c>
       <c r="L315" s="17" t="n">
-        <v>432</v>
+        <v>328</v>
       </c>
       <c r="M315" s="17" t="inlineStr">
         <is>
@@ -24068,7 +24068,7 @@
         </is>
       </c>
       <c r="L316" s="17" t="n">
-        <v>640</v>
+        <v>534</v>
       </c>
       <c r="M316" s="17" t="inlineStr">
         <is>
@@ -24141,7 +24141,7 @@
         </is>
       </c>
       <c r="L317" s="17" t="n">
-        <v>287</v>
+        <v>495</v>
       </c>
       <c r="M317" s="17" t="inlineStr">
         <is>
@@ -24214,7 +24214,7 @@
         </is>
       </c>
       <c r="L318" s="17" t="n">
-        <v>496</v>
+        <v>579</v>
       </c>
       <c r="M318" s="17" t="inlineStr">
         <is>

</xml_diff>